<commit_message>
Update INDOPROSTIME sample1 reference to match current extraction
Per user decision, the extraction result is the source of truth for this
sample: invoice/on-board dates as YYYY-MON-DD text, consignee
"HARDASES ABADI INDONESIA,.PT", description "FREIGHT CHARGE (USD 23.54)",
volume "1.6 KG", vessel "CX 777". learned_configs.json score updated.

Regression: 49/49 samples at 100% (with Tesseract installed locally).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_samples/INDOPROSTIME/sample1_ref.xlsx
+++ b/test_samples/INDOPROSTIME/sample1_ref.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DWIHARTA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DWIHARTA" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -609,7 +609,7 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>02 Sep 2026</t>
+          <t>2026-SEP-02</t>
         </is>
       </c>
       <c r="B2" s="0" t="n">
@@ -622,12 +622,12 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t>PT. HARDASES ABADI INDONESIA</t>
+          <t>HARDASES ABADI INDONESIA,.PT</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
         <is>
-          <t>FREIGHT CHARGE</t>
+          <t>FREIGHT CHARGE (USD 23.54)</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
@@ -645,7 +645,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>01 Sep 2026</t>
+          <t>2026-SEP-01</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -668,12 +668,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="N2" s="0" t="n">
-        <v>1.6</v>
+      <c r="N2" s="0" t="inlineStr">
+        <is>
+          <t>1.6 KG</t>
+        </is>
       </c>
       <c r="O2" s="0" t="inlineStr">
         <is>
-          <t>CX 777/01092026</t>
+          <t>CX 777</t>
         </is>
       </c>
       <c r="P2" s="0" t="inlineStr">
@@ -712,9 +714,6 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="Q12" s="1" t="n"/>
     </row>

</xml_diff>